<commit_message>
update bootstrap output files
</commit_message>
<xml_diff>
--- a/CPRD Raw Analysis/Results/Output_costs_Raw-Unadjusted_Boot.xlsx
+++ b/CPRD Raw Analysis/Results/Output_costs_Raw-Unadjusted_Boot.xlsx
@@ -377,10 +377,10 @@
         <v>1072.132</v>
       </c>
       <c r="B2">
-        <v>1059.613</v>
+        <v>1060.137</v>
       </c>
       <c r="C2">
-        <v>1085.577</v>
+        <v>1084.188</v>
       </c>
     </row>
   </sheetData>
@@ -415,10 +415,10 @@
         <v>1089.035</v>
       </c>
       <c r="B2">
-        <v>1077.07</v>
+        <v>1077.344</v>
       </c>
       <c r="C2">
-        <v>1101.647</v>
+        <v>1100.79</v>
       </c>
     </row>
   </sheetData>

</xml_diff>